<commit_message>
Added Option 5 Student lookup and transaction analysis
</commit_message>
<xml_diff>
--- a/docs/tblStudent.xlsx
+++ b/docs/tblStudent.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\jadiDashboard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C162974-90EE-435B-BBAF-57C1E2C6A7E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F40B80-BDED-4E2C-97E1-76505512D760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2620" yWindow="2620" windowWidth="14400" windowHeight="7810" xr2:uid="{96F36FC2-362B-4770-BF65-158E8C9DB39E}"/>
+    <workbookView xWindow="4190" yWindow="860" windowWidth="14400" windowHeight="7810" xr2:uid="{96F36FC2-362B-4770-BF65-158E8C9DB39E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>Column</t>
   </si>
@@ -48,6 +48,93 @@
   </si>
   <si>
     <t>Alias</t>
+  </si>
+  <si>
+    <t>idnumber</t>
+  </si>
+  <si>
+    <t>lastname</t>
+  </si>
+  <si>
+    <t>firstname</t>
+  </si>
+  <si>
+    <t>midname</t>
+  </si>
+  <si>
+    <t>AccountBalance</t>
+  </si>
+  <si>
+    <t>CNP</t>
+  </si>
+  <si>
+    <t>LastCleared</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>StateCode</t>
+  </si>
+  <si>
+    <t>Zipcode</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>ClearedCurrentSession</t>
+  </si>
+  <si>
+    <t>ClearedOn</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Student ID Number </t>
+  </si>
+  <si>
+    <t>Student Last Name</t>
+  </si>
+  <si>
+    <t>Student First Name</t>
+  </si>
+  <si>
+    <t>Student Middle Name (If available)</t>
+  </si>
+  <si>
+    <t>Current balance owed</t>
+  </si>
+  <si>
+    <t>Credits Not Posted (Not reliable)</t>
+  </si>
+  <si>
+    <t>Last Semester student attended</t>
+  </si>
+  <si>
+    <t>Street Address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">State or Province </t>
+  </si>
+  <si>
+    <t>Postal Code</t>
+  </si>
+  <si>
+    <t>Telephone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value = 1 when student is financially cleared for Semester in &lt;LastCleared&gt; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">String containing the date student was financially cleared </t>
+  </si>
+  <si>
+    <t>Country of Residence</t>
   </si>
 </sst>
 </file>
@@ -419,10 +506,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEADB764-BB07-487D-9A45-F7F09656D0A9}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.1796875" customWidth="1"/>
+    <col min="1" max="1" width="20.453125" customWidth="1"/>
     <col min="2" max="2" width="68.26953125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -437,6 +524,126 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>